<commit_message>
refactor: RemoteDataManager 코드 정리. (로직 복구) refactor: MobileApplication 코드 정리. feature: ShopProductDaily 일일 5개 선택 기능 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/ShopTable.xlsx
+++ b/input/Domains/Game/ShopTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72D51A64-8670-CA45-A0F8-9901E5C51792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BEBC48B-815F-1B43-B01A-01C4A1175866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46300" yWindow="120" windowWidth="27700" windowHeight="16880" activeTab="3" xr2:uid="{A79F8533-37C3-E444-AEC4-352841701A9E}"/>
+    <workbookView xWindow="40660" yWindow="-200" windowWidth="27700" windowHeight="16880" activeTab="1" xr2:uid="{A79F8533-37C3-E444-AEC4-352841701A9E}"/>
   </bookViews>
   <sheets>
     <sheet name="PURCHASE" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="95">
   <si>
     <t>internalProductId</t>
   </si>
@@ -155,28 +155,16 @@
     <t>상품 ID</t>
   </si>
   <si>
-    <t>shop_001_free</t>
-  </si>
-  <si>
     <t>FREE</t>
   </si>
   <si>
     <t>reward_shop_001</t>
   </si>
   <si>
-    <t>shop_001_ads</t>
-  </si>
-  <si>
     <t>ADS</t>
   </si>
   <si>
-    <t>shop_001_x01</t>
-  </si>
-  <si>
     <t>JEWEL</t>
-  </si>
-  <si>
-    <t>shop_001_x10</t>
   </si>
   <si>
     <t>maxCount</t>
@@ -191,14 +179,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>shop_treasure_x01</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>shop_treasure_x10</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>shop_noads_month</t>
   </si>
   <si>
@@ -312,6 +292,62 @@
   <si>
     <t>shop_jewel_1000</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>shop_treasure_001</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>shop_treasure_010</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>shop_daily_free</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>shop_daily_ads</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>shop_daily_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>shop_daily_002</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>float</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>selectRate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>shop_daily_003</t>
+  </si>
+  <si>
+    <t>shop_daily_004</t>
+  </si>
+  <si>
+    <t>shop_daily_005</t>
+  </si>
+  <si>
+    <t>shop_daily_006</t>
+  </si>
+  <si>
+    <t>shop_daily_007</t>
+  </si>
+  <si>
+    <t>shop_daily_008</t>
+  </si>
+  <si>
+    <t>shop_daily_009</t>
+  </si>
+  <si>
+    <t>shop_daily_010</t>
   </si>
 </sst>
 </file>
@@ -802,7 +838,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>19</v>
@@ -822,7 +858,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>22</v>
@@ -844,7 +880,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>26</v>
@@ -858,7 +894,7 @@
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="H7" s="1"/>
     </row>
@@ -870,10 +906,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56687F69-CC51-6347-8247-334F985F2F67}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -895,8 +935,11 @@
       <c r="G1" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -918,8 +961,11 @@
       <c r="G2" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -930,7 +976,7 @@
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
         <v>36</v>
       </c>
@@ -941,19 +987,19 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F5" s="1">
         <v>1</v>
@@ -961,20 +1007,23 @@
       <c r="G5" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5" s="1">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="1" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D6" s="1">
         <v>0</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F6" s="1">
         <v>1</v>
@@ -982,48 +1031,259 @@
       <c r="G6" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="H6" s="1">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D7" s="1">
         <v>100</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F7" s="1">
         <v>1</v>
       </c>
       <c r="G7" s="1">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>1</v>
+      </c>
+      <c r="H7" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" s="1" t="s">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D8" s="1">
         <v>1000</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F8" s="1">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G8" s="1">
-        <v>-1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H8" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1000</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="1">
+        <v>1</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1</v>
+      </c>
+      <c r="H9" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1000</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1</v>
+      </c>
+      <c r="H10" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1000</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1</v>
+      </c>
+      <c r="G11" s="1">
+        <v>1</v>
+      </c>
+      <c r="H11" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1000</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1</v>
+      </c>
+      <c r="H12" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1000</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="1">
+        <v>1</v>
+      </c>
+      <c r="G13" s="1">
+        <v>1</v>
+      </c>
+      <c r="H13" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="1">
+        <v>1000</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="1">
+        <v>1</v>
+      </c>
+      <c r="G14" s="1">
+        <v>1</v>
+      </c>
+      <c r="H14" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="1">
+        <v>1000</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="1">
+        <v>1</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1</v>
+      </c>
+      <c r="H15" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1000</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16" s="1">
+        <v>1</v>
+      </c>
+      <c r="G16" s="1">
+        <v>1</v>
+      </c>
+      <c r="H16" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1035,6 +1295,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D801677-7933-234D-87BC-066B152A0555}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
@@ -1056,7 +1320,7 @@
         <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -1079,7 +1343,7 @@
         <v>35</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1106,17 +1370,17 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F5" s="1">
         <v>1</v>
@@ -1127,17 +1391,17 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="1" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D6" s="1">
         <v>100</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F6" s="1">
         <v>1</v>
@@ -1148,17 +1412,17 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="1" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D7" s="1">
         <v>1000</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F7" s="1">
         <v>11</v>
@@ -1230,21 +1494,21 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>25</v>
@@ -1252,11 +1516,11 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D7" s="1"/>
     </row>
@@ -1291,7 +1555,7 @@
         <v>1</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1311,7 +1575,7 @@
         <v>8</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1336,15 +1600,15 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F5" s="1">
         <v>5</v>
@@ -1352,17 +1616,17 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D6" s="1">
         <v>500</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F6" s="1">
         <v>-1</v>
@@ -1370,17 +1634,17 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D7" s="1">
         <v>1500</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F7" s="1">
         <v>-1</v>
@@ -1402,22 +1666,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>32</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1428,7 +1692,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>8</v>
@@ -1437,7 +1701,7 @@
         <v>35</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1445,7 +1709,7 @@
         <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1454,19 +1718,19 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F4" s="1"/>
     </row>
@@ -1478,10 +1742,10 @@
         <v>22</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E5" s="1">
         <v>1000</v>
@@ -1501,7 +1765,7 @@
         <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="E6" s="1">
         <v>1</v>
@@ -1521,7 +1785,7 @@
         <v>23</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E7" s="1">
         <v>1</v>
@@ -1535,13 +1799,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E8" s="1">
         <v>1000</v>
@@ -1555,13 +1819,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E9" s="1">
         <v>1</v>
@@ -1575,13 +1839,13 @@
         <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E10" s="1">
         <v>1</v>
@@ -1595,13 +1859,13 @@
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E11" s="1">
         <v>1</v>
@@ -1615,13 +1879,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E12" s="1">
         <v>1</v>
@@ -1635,13 +1899,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E13" s="1">
         <v>1</v>

</xml_diff>

<commit_message>
feature: 구매 복원 기능 추가. init session function 삭제.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/ShopTable.xlsx
+++ b/input/Domains/Game/ShopTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BEBC48B-815F-1B43-B01A-01C4A1175866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0B583F-C3CA-0F4B-A117-84C60D0CC51E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40660" yWindow="-200" windowWidth="27700" windowHeight="16880" activeTab="1" xr2:uid="{A79F8533-37C3-E444-AEC4-352841701A9E}"/>
+    <workbookView xWindow="4220" yWindow="1840" windowWidth="27700" windowHeight="16880" xr2:uid="{A79F8533-37C3-E444-AEC4-352841701A9E}"/>
   </bookViews>
   <sheets>
     <sheet name="PURCHASE" sheetId="1" r:id="rId1"/>
@@ -744,8 +744,9 @@
   <cols>
     <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
     <col min="7" max="7" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">

</xml_diff>

<commit_message>
refactor: achieve storage state 적용 및 리팩토링.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/ShopTable.xlsx
+++ b/input/Domains/Game/ShopTable.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04C3B3C-CB0A-5740-8CE2-FBE241DCB423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BDF7EAA-1BD4-3A41-9F53-D3B1A68221D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4580" yWindow="2120" windowWidth="27700" windowHeight="16880" xr2:uid="{A79F8533-37C3-E444-AEC4-352841701A9E}"/>
+    <workbookView xWindow="4580" yWindow="2120" windowWidth="27700" windowHeight="16880" activeTab="4" xr2:uid="{A79F8533-37C3-E444-AEC4-352841701A9E}"/>
   </bookViews>
   <sheets>
     <sheet name="SHOP_CATALOG" sheetId="7" r:id="rId1"/>
-    <sheet name="SHOP_DAILY" sheetId="2" r:id="rId2"/>
-    <sheet name="SHOP_EVENT" sheetId="8" r:id="rId3"/>
-    <sheet name="SHOP_CHEST" sheetId="3" r:id="rId4"/>
-    <sheet name="SHOP_PURCHASE" sheetId="4" r:id="rId5"/>
-    <sheet name="SHOP_GOLD" sheetId="5" r:id="rId6"/>
-    <sheet name="PURCHASE" sheetId="1" r:id="rId7"/>
-    <sheet name="REWARD@SHOP" sheetId="6" r:id="rId8"/>
+    <sheet name="SHOP_CATALOG_CHEST" sheetId="9" r:id="rId2"/>
+    <sheet name="SHOP_DAILY" sheetId="2" r:id="rId3"/>
+    <sheet name="SHOP_EVENT" sheetId="8" r:id="rId4"/>
+    <sheet name="SHOP_CHEST" sheetId="3" r:id="rId5"/>
+    <sheet name="SHOP_PURCHASE" sheetId="4" r:id="rId6"/>
+    <sheet name="SHOP_GOLD" sheetId="5" r:id="rId7"/>
+    <sheet name="PURCHASE" sheetId="1" r:id="rId8"/>
+    <sheet name="REWARD@SHOP" sheetId="6" r:id="rId9"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="123">
   <si>
     <t>internalProductId</t>
   </si>
@@ -445,6 +446,18 @@
   </si>
   <si>
     <t>enum:SHOP_CATALOG_TYPE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gainExp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>exp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>level</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -964,6 +977,198 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A046F419-4246-714D-A1BD-91A2DDA55701}">
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15">
+        <v>11</v>
+      </c>
+      <c r="B15">
+        <v>5500</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16">
+        <v>12</v>
+      </c>
+      <c r="B16">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17">
+        <v>13</v>
+      </c>
+      <c r="B17">
+        <v>6500</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18">
+        <v>14</v>
+      </c>
+      <c r="B18">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19">
+        <v>15</v>
+      </c>
+      <c r="B19">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20">
+        <v>16</v>
+      </c>
+      <c r="B20">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21">
+        <v>17</v>
+      </c>
+      <c r="B21">
+        <v>8500</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22">
+        <v>18</v>
+      </c>
+      <c r="B22">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23">
+        <v>19</v>
+      </c>
+      <c r="B23">
+        <v>9500</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24">
+        <v>20</v>
+      </c>
+      <c r="B24">
+        <v>-1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56687F69-CC51-6347-8247-334F985F2F67}">
   <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
@@ -1495,7 +1700,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D30A11D-6558-A646-A0EF-457EBBC26B2A}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
@@ -1624,16 +1829,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D801677-7933-234D-87BC-066B152A0555}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -1655,8 +1860,11 @@
       <c r="G1" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1678,8 +1886,11 @@
       <c r="G2" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1690,7 +1901,7 @@
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
         <v>35</v>
       </c>
@@ -1701,7 +1912,7 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
         <v>42</v>
       </c>
@@ -1721,8 +1932,11 @@
       <c r="G5" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="H5" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="1" t="s">
         <v>78</v>
       </c>
@@ -1742,8 +1956,11 @@
       <c r="G6" s="1">
         <v>-1</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="H6" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
         <v>79</v>
       </c>
@@ -1762,6 +1979,9 @@
       </c>
       <c r="G7" s="1">
         <v>-1</v>
+      </c>
+      <c r="H7" s="1">
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -1770,7 +1990,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{224A3DC9-4299-B34F-A393-B87C3C3DFA12}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
@@ -1863,7 +2083,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79EDF6A7-3BA9-C14F-AA9E-54512EB4B167}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
@@ -1990,7 +2210,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30FDEFE6-D501-CD4D-AE74-F5C615598DFE}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
@@ -2131,7 +2351,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FCA191E-CD52-EA4F-A8D1-26E811B9CEBA}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>

</xml_diff>

<commit_message>
feature: daily shop 기능 구현.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/ShopTable.xlsx
+++ b/input/Domains/Game/ShopTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2785AB46-3539-104C-87AB-C0FC3E158E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D6E939-9BE2-BF4E-8204-A7A4A7658C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4580" yWindow="2120" windowWidth="31280" windowHeight="16880" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4580" yWindow="2120" windowWidth="31280" windowHeight="16880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SHOP_CATALOG" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="126">
   <si>
     <t>catalog_type</t>
   </si>
@@ -129,99 +129,105 @@
     <t>reward_group_id</t>
   </si>
   <si>
+    <t>amount_min</t>
+  </si>
+  <si>
+    <t>amount_max</t>
+  </si>
+  <si>
+    <t>max_count</t>
+  </si>
+  <si>
+    <t>select_rate</t>
+  </si>
+  <si>
+    <t>discount_rate10_per</t>
+  </si>
+  <si>
+    <t>discount_rate20_per</t>
+  </si>
+  <si>
+    <t>discount_rate30_per</t>
+  </si>
+  <si>
+    <t>discount_rate50_per</t>
+  </si>
+  <si>
+    <t>CURRENCY_TYPE</t>
+  </si>
+  <si>
+    <t>float</t>
+  </si>
+  <si>
+    <t>상품 ID</t>
+  </si>
+  <si>
+    <t>shop_daily_free</t>
+  </si>
+  <si>
+    <t>FREE</t>
+  </si>
+  <si>
+    <t>shop_daily_ads</t>
+  </si>
+  <si>
+    <t>ADS</t>
+  </si>
+  <si>
+    <t>shop_daily_001</t>
+  </si>
+  <si>
+    <t>JEWEL</t>
+  </si>
+  <si>
+    <t>shop_daily_002</t>
+  </si>
+  <si>
+    <t>shop_daily_003</t>
+  </si>
+  <si>
+    <t>shop_daily_004</t>
+  </si>
+  <si>
+    <t>shop_daily_005</t>
+  </si>
+  <si>
+    <t>shop_daily_006</t>
+  </si>
+  <si>
+    <t>shop_daily_007</t>
+  </si>
+  <si>
+    <t>shop_daily_008</t>
+  </si>
+  <si>
+    <t>shop_daily_009</t>
+  </si>
+  <si>
+    <t>shop_daily_010</t>
+  </si>
+  <si>
+    <t>start_time</t>
+  </si>
+  <si>
+    <t>end_time</t>
+  </si>
+  <si>
+    <t>CDateTime</t>
+  </si>
+  <si>
+    <t>shop_event_001</t>
+  </si>
+  <si>
+    <t>shop_event_002</t>
+  </si>
+  <si>
+    <t>chest_type</t>
+  </si>
+  <si>
     <t>amount</t>
   </si>
   <si>
-    <t>max_count</t>
-  </si>
-  <si>
-    <t>select_rate</t>
-  </si>
-  <si>
-    <t>discount_rate10_per</t>
-  </si>
-  <si>
-    <t>discount_rate20_per</t>
-  </si>
-  <si>
-    <t>discount_rate30_per</t>
-  </si>
-  <si>
-    <t>discount_rate50_per</t>
-  </si>
-  <si>
-    <t>CURRENCY_TYPE</t>
-  </si>
-  <si>
-    <t>float</t>
-  </si>
-  <si>
-    <t>상품 ID</t>
-  </si>
-  <si>
-    <t>shop_daily_free</t>
-  </si>
-  <si>
-    <t>FREE</t>
-  </si>
-  <si>
-    <t>shop_daily_ads</t>
-  </si>
-  <si>
-    <t>ADS</t>
-  </si>
-  <si>
-    <t>shop_daily_001</t>
-  </si>
-  <si>
-    <t>JEWEL</t>
-  </si>
-  <si>
-    <t>shop_daily_002</t>
-  </si>
-  <si>
-    <t>shop_daily_003</t>
-  </si>
-  <si>
-    <t>shop_daily_004</t>
-  </si>
-  <si>
-    <t>shop_daily_005</t>
-  </si>
-  <si>
-    <t>shop_daily_006</t>
-  </si>
-  <si>
-    <t>shop_daily_007</t>
-  </si>
-  <si>
-    <t>shop_daily_008</t>
-  </si>
-  <si>
-    <t>shop_daily_009</t>
-  </si>
-  <si>
-    <t>shop_daily_010</t>
-  </si>
-  <si>
-    <t>start_time</t>
-  </si>
-  <si>
-    <t>end_time</t>
-  </si>
-  <si>
-    <t>CDateTime</t>
-  </si>
-  <si>
-    <t>shop_event_001</t>
-  </si>
-  <si>
-    <t>shop_event_002</t>
-  </si>
-  <si>
-    <t>chest_type</t>
-  </si>
-  <si>
     <t>SHOP_PRODUCT_CHEST_TYPE</t>
   </si>
   <si>
@@ -273,6 +279,9 @@
     <t>shop_gold_001_ads</t>
   </si>
   <si>
+    <t>shop_gold_001</t>
+  </si>
+  <si>
     <t>shop_gold_002</t>
   </si>
   <si>
@@ -396,12 +405,7 @@
     <t>CARD</t>
   </si>
   <si>
-    <t>shop_gold_001</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>item_card_001</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -878,7 +882,7 @@
         <v>18</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1488,7 +1492,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1496,7 +1500,7 @@
     <col min="9" max="12" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" t="s">
         <v>29</v>
       </c>
@@ -1533,8 +1537,11 @@
       <c r="L1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1542,7 +1549,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -1557,37 +1564,40 @@
         <v>8</v>
       </c>
       <c r="H2" t="s">
-        <v>41</v>
+        <v>8</v>
       </c>
       <c r="I2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>42</v>
+      </c>
+      <c r="M2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1602,15 +1612,18 @@
         <v>1</v>
       </c>
       <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
         <v>-1</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -1622,18 +1635,21 @@
         <v>1</v>
       </c>
       <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
         <v>3</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>-1</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D7">
         <v>100</v>
@@ -1648,27 +1664,30 @@
         <v>1</v>
       </c>
       <c r="H7">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="J7">
+        <v>50</v>
+      </c>
+      <c r="K7">
         <v>25</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>15</v>
       </c>
-      <c r="L7">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+      <c r="M7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
         <v>49</v>
-      </c>
-      <c r="C8" t="s">
-        <v>48</v>
       </c>
       <c r="D8">
         <v>1000</v>
@@ -1680,30 +1699,33 @@
         <v>1</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H8">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="J8">
+        <v>50</v>
+      </c>
+      <c r="K8">
         <v>25</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>15</v>
       </c>
-      <c r="L8">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+      <c r="M8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D9">
         <v>1000</v>
@@ -1715,30 +1737,33 @@
         <v>1</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H9">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="J9">
+        <v>50</v>
+      </c>
+      <c r="K9">
         <v>25</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>15</v>
       </c>
-      <c r="L9">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+      <c r="M9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D10">
         <v>1000</v>
@@ -1750,30 +1775,33 @@
         <v>1</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H10">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="J10">
+        <v>50</v>
+      </c>
+      <c r="K10">
         <v>25</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>15</v>
       </c>
-      <c r="L10">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+      <c r="M10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D11">
         <v>1000</v>
@@ -1785,30 +1813,33 @@
         <v>1</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H11">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I11">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="J11">
+        <v>50</v>
+      </c>
+      <c r="K11">
         <v>25</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>15</v>
       </c>
-      <c r="L11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
+      <c r="M11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D12">
         <v>1000</v>
@@ -1820,30 +1851,33 @@
         <v>1</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H12">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I12">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="J12">
+        <v>50</v>
+      </c>
+      <c r="K12">
         <v>25</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>15</v>
       </c>
-      <c r="L12">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
+      <c r="M12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D13">
         <v>1000</v>
@@ -1855,30 +1889,33 @@
         <v>1</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H13">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I13">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="J13">
+        <v>50</v>
+      </c>
+      <c r="K13">
         <v>25</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>15</v>
       </c>
-      <c r="L13">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
+      <c r="M13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D14">
         <v>1000</v>
@@ -1890,30 +1927,33 @@
         <v>1</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H14">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I14">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="J14">
+        <v>50</v>
+      </c>
+      <c r="K14">
         <v>25</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>15</v>
       </c>
-      <c r="L14">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
+      <c r="M14">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D15">
         <v>1000</v>
@@ -1925,30 +1965,33 @@
         <v>1</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H15">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I15">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="J15">
+        <v>50</v>
+      </c>
+      <c r="K15">
         <v>25</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>15</v>
       </c>
-      <c r="L15">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12">
+      <c r="M15">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D16">
         <v>1000</v>
@@ -1960,21 +2003,24 @@
         <v>1</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H16">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I16">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="J16">
+        <v>50</v>
+      </c>
+      <c r="K16">
         <v>25</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>15</v>
       </c>
-      <c r="L16">
+      <c r="M16">
         <v>10</v>
       </c>
     </row>
@@ -2011,10 +2057,10 @@
         <v>32</v>
       </c>
       <c r="F1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -2025,7 +2071,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -2034,10 +2080,10 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -2047,15 +2093,15 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D5">
         <v>100</v>
@@ -2072,10 +2118,10 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D6">
         <v>100</v>
@@ -2111,7 +2157,7 @@
         <v>29</v>
       </c>
       <c r="B1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -2123,10 +2169,10 @@
         <v>31</v>
       </c>
       <c r="F1" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="G1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -2134,13 +2180,13 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -2159,18 +2205,18 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -2184,13 +2230,13 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E6">
         <v>100</v>
@@ -2204,13 +2250,13 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E7">
         <v>1000</v>
@@ -2245,10 +2291,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2272,37 +2318,37 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -2337,7 +2383,7 @@
         <v>32</v>
       </c>
       <c r="F1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2348,7 +2394,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -2367,15 +2413,15 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
         <v>28</v>
@@ -2386,10 +2432,10 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>122</v>
+        <v>83</v>
       </c>
       <c r="C6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D6">
         <v>500</v>
@@ -2403,10 +2449,10 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D7">
         <v>1500</v>
@@ -2437,22 +2483,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B1" t="s">
         <v>32</v>
       </c>
       <c r="C1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2463,10 +2509,10 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
@@ -2482,73 +2528,73 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C7" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -2567,22 +2613,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B1" t="s">
         <v>32</v>
       </c>
       <c r="C1" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E1" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="F1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2593,7 +2639,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -2602,7 +2648,7 @@
         <v>8</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2610,24 +2656,24 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2635,13 +2681,13 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E5">
         <v>1000</v>
@@ -2655,13 +2701,13 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C6" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -2675,13 +2721,13 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D7" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2695,13 +2741,13 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C8" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D8" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E8">
         <v>1000</v>
@@ -2715,13 +2761,13 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C9" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2735,13 +2781,13 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C10" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D10" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2755,13 +2801,13 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C11" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D11" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2778,10 +2824,10 @@
         <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2798,10 +2844,10 @@
         <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E13">
         <v>1</v>

</xml_diff>

<commit_message>
feature: gold shop 구현. docs: 스킬 문저 정리. refactor: inventory message 정리.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/ShopTable.xlsx
+++ b/input/Domains/Game/ShopTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08851DED-D800-E94A-AAF1-1852AE025D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADB4905-DC06-5B47-8102-8FE6FDF1BF57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4580" yWindow="2120" windowWidth="31280" windowHeight="16880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4580" yWindow="2120" windowWidth="31280" windowHeight="16880" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SHOP_CATALOG" sheetId="1" r:id="rId1"/>
@@ -2442,7 +2442,7 @@
         <v>49</v>
       </c>
       <c r="D6">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
         <v>28</v>
@@ -2459,7 +2459,7 @@
         <v>49</v>
       </c>
       <c r="D7">
-        <v>1500</v>
+        <v>150</v>
       </c>
       <c r="E7" t="s">
         <v>28</v>

</xml_diff>